<commit_message>
last updates and pushed last versions to repos
</commit_message>
<xml_diff>
--- a/006_Can_SapAriba_eBay_Performer/Data/eBayPerformerConfig.xlsx
+++ b/006_Can_SapAriba_eBay_Performer/Data/eBayPerformerConfig.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grmusarpadev11\Desktop\linktera\YALCIN\bayer\content\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\1files\uipath\projects\006_Can_SapAriba_eBay\006_Can_SapAriba_eBay_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A28D5E-5D77-4A5E-BE6A-4BE883B877D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA076A63-65B6-49F1-BD98-8F89F7E4770D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13425" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="13305" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
   <si>
     <t>Name</t>
   </si>
@@ -165,23 +165,116 @@
     <t>SapAribaUrl</t>
   </si>
   <si>
-    <t>GMCAN_FINANCE_AR</t>
-  </si>
-  <si>
     <t>SupportTeam</t>
   </si>
   <si>
-    <t>testmailaddress</t>
-  </si>
-  <si>
-    <t>eBay_SAP_Ariba</t>
+    <t>url of sap ariba</t>
+  </si>
+  <si>
+    <t>Canada_AR_SupportTeam</t>
+  </si>
+  <si>
+    <t>In the library the input must be separated by ";"</t>
+  </si>
+  <si>
+    <t>AzureTenantID</t>
+  </si>
+  <si>
+    <t>_CADGRM.SAP_TenantID</t>
+  </si>
+  <si>
+    <t>Azure Tenant ID</t>
+  </si>
+  <si>
+    <t>AzureAppID</t>
+  </si>
+  <si>
+    <t>_CADGRM.SAP_AppID</t>
+  </si>
+  <si>
+    <t>Azure Application ID</t>
+  </si>
+  <si>
+    <t>SiteURL</t>
+  </si>
+  <si>
+    <t>CADGRM.SAP_SiteUrl</t>
+  </si>
+  <si>
+    <t>Site URL of SharePoint site</t>
+  </si>
+  <si>
+    <t>DriveName</t>
+  </si>
+  <si>
+    <t>CADGRM.SAP.DriveName</t>
+  </si>
+  <si>
+    <t>DriveName of the SharePoint site</t>
+  </si>
+  <si>
+    <t>SharePointSubFolder</t>
+  </si>
+  <si>
+    <t>Canada_AR_SharepointFolder</t>
+  </si>
+  <si>
+    <t>SharePoint subfolder</t>
+  </si>
+  <si>
+    <t>bulent.yarbasi@linktera.com</t>
+  </si>
+  <si>
+    <t>Credentials</t>
+  </si>
+  <si>
+    <t>SapAribaCredentialName</t>
+  </si>
+  <si>
+    <t>Can_SapAriba_Mars_Credentials</t>
+  </si>
+  <si>
+    <t>AppSecretCredentialName</t>
+  </si>
+  <si>
+    <t>_CADGRM.SAP_AppSecret</t>
+  </si>
+  <si>
+    <t>Office365CredentialsName</t>
+  </si>
+  <si>
+    <t>CADGRM.SAP.Office365Credentials</t>
+  </si>
+  <si>
+    <t>SMEs</t>
+  </si>
+  <si>
+    <t>outputFolderPath</t>
+  </si>
+  <si>
+    <t>C:\1files\uipath\can_ar_ariba\ebay\invoice_reports\</t>
+  </si>
+  <si>
+    <t>ClientName</t>
+  </si>
+  <si>
+    <t>SapAribaEbay</t>
+  </si>
+  <si>
+    <t>CanSapAribaEbay_Queue</t>
+  </si>
+  <si>
+    <t>customerNameSAP</t>
+  </si>
+  <si>
+    <t>eBay, Inc.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -202,6 +295,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -226,7 +325,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -236,6 +335,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -550,7 +650,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
+  <dimension ref="A1:Z997"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -598,7 +698,7 @@
         <v>24</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>22</v>
@@ -607,9 +707,6 @@
     <row r="3" spans="1:26" ht="45">
       <c r="A3" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>46</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>32</v>
@@ -628,39 +725,85 @@
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" t="s">
-        <v>48</v>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>67</v>
+      </c>
+      <c r="B10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="15" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+    </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" ht="14.25" customHeight="1"/>
-    <row r="18" ht="14.25" customHeight="1"/>
-    <row r="19" ht="14.25" customHeight="1"/>
-    <row r="20" ht="14.25" customHeight="1"/>
-    <row r="21" ht="14.25" customHeight="1"/>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
-    <row r="24" ht="14.25" customHeight="1"/>
-    <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
-    <row r="32" ht="14.25" customHeight="1"/>
+    <row r="17" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="21" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -1626,7 +1769,6 @@
     <row r="995" ht="14.25" customHeight="1"/>
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2794,7 +2936,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z999"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
@@ -2847,16 +2989,76 @@
       <c r="B2" t="s">
         <v>44</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A3" t="s">
         <v>46</v>
       </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="3" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="5" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="4" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D8" t="s">
+        <v>64</v>
+      </c>
+    </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -3848,7 +4050,6 @@
     <row r="997" ht="14.25" customHeight="1"/>
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
-    <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>